<commit_message>
Remove temporary Excel lock file
</commit_message>
<xml_diff>
--- a/data/demo_data.xlsx
+++ b/data/demo_data.xlsx
@@ -10,14 +10,14 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FECBB9A-076B-F049-8F7E-3B9B7336B3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16200" activeTab="2" xr2:uid="{E3A46B07-642E-F742-AB13-04A6A75806A3}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{E3A46B07-642E-F742-AB13-04A6A75806A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Clients" sheetId="1" r:id="rId1"/>
     <sheet name="Pets" sheetId="2" r:id="rId2"/>
     <sheet name="Visits" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>